<commit_message>
fix: enable query for job details based on code and adjust Playwright config for CI
</commit_message>
<xml_diff>
--- a/docs/test-report.xlsx
+++ b/docs/test-report.xlsx
@@ -425,7 +425,7 @@
         <v>Passed</v>
       </c>
       <c r="B3">
-        <v>111</v>
+        <v>115</v>
       </c>
     </row>
     <row r="4">
@@ -433,7 +433,7 @@
         <v>Failed</v>
       </c>
       <c r="B4">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -441,7 +441,7 @@
         <v>Skipped</v>
       </c>
       <c r="B5">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
@@ -449,7 +449,7 @@
         <v>Pass Rate</v>
       </c>
       <c r="B6" t="str">
-        <v>98%</v>
+        <v>100%</v>
       </c>
     </row>
     <row r="7">
@@ -457,7 +457,7 @@
         <v>Run Date</v>
       </c>
       <c r="B7" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="8">
@@ -465,7 +465,7 @@
         <v>Total Duration</v>
       </c>
       <c r="B8" t="str">
-        <v>4.4 min</v>
+        <v>4.8 min</v>
       </c>
     </row>
     <row r="9">
@@ -548,13 +548,13 @@
         <v>PASSED</v>
       </c>
       <c r="F2">
-        <v>4.8</v>
+        <v>16.3</v>
       </c>
       <c r="G2" t="str">
         <v>chromium</v>
       </c>
       <c r="H2" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="3">
@@ -574,13 +574,13 @@
         <v>PASSED</v>
       </c>
       <c r="F3">
-        <v>5.2</v>
+        <v>16</v>
       </c>
       <c r="G3" t="str">
         <v>chromium</v>
       </c>
       <c r="H3" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="4">
@@ -600,13 +600,13 @@
         <v>PASSED</v>
       </c>
       <c r="F4">
-        <v>4.2</v>
+        <v>4.1</v>
       </c>
       <c r="G4" t="str">
         <v>chromium</v>
       </c>
       <c r="H4" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="5">
@@ -626,13 +626,13 @@
         <v>PASSED</v>
       </c>
       <c r="F5">
-        <v>4.2</v>
+        <v>4.1</v>
       </c>
       <c r="G5" t="str">
         <v>chromium</v>
       </c>
       <c r="H5" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="6">
@@ -652,13 +652,13 @@
         <v>PASSED</v>
       </c>
       <c r="F6">
-        <v>3.8</v>
+        <v>4</v>
       </c>
       <c r="G6" t="str">
         <v>chromium</v>
       </c>
       <c r="H6" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="7">
@@ -678,13 +678,13 @@
         <v>PASSED</v>
       </c>
       <c r="F7">
-        <v>4</v>
+        <v>3.8</v>
       </c>
       <c r="G7" t="str">
         <v>chromium</v>
       </c>
       <c r="H7" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="8">
@@ -704,13 +704,13 @@
         <v>PASSED</v>
       </c>
       <c r="F8">
-        <v>4</v>
+        <v>4.5</v>
       </c>
       <c r="G8" t="str">
         <v>chromium</v>
       </c>
       <c r="H8" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="9">
@@ -730,13 +730,13 @@
         <v>PASSED</v>
       </c>
       <c r="F9">
-        <v>3.7</v>
+        <v>4.4</v>
       </c>
       <c r="G9" t="str">
         <v>chromium</v>
       </c>
       <c r="H9" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="10">
@@ -756,13 +756,13 @@
         <v>PASSED</v>
       </c>
       <c r="F10">
-        <v>4</v>
+        <v>4.1</v>
       </c>
       <c r="G10" t="str">
         <v>chromium</v>
       </c>
       <c r="H10" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="11">
@@ -782,13 +782,13 @@
         <v>PASSED</v>
       </c>
       <c r="F11">
-        <v>4</v>
+        <v>4.1</v>
       </c>
       <c r="G11" t="str">
         <v>chromium</v>
       </c>
       <c r="H11" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="12">
@@ -808,13 +808,13 @@
         <v>PASSED</v>
       </c>
       <c r="F12">
-        <v>3.8</v>
+        <v>4.5</v>
       </c>
       <c r="G12" t="str">
         <v>chromium</v>
       </c>
       <c r="H12" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="13">
@@ -834,13 +834,13 @@
         <v>PASSED</v>
       </c>
       <c r="F13">
-        <v>3.9</v>
+        <v>4.5</v>
       </c>
       <c r="G13" t="str">
         <v>chromium</v>
       </c>
       <c r="H13" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="14">
@@ -860,13 +860,13 @@
         <v>PASSED</v>
       </c>
       <c r="F14">
-        <v>3.8</v>
+        <v>5.5</v>
       </c>
       <c r="G14" t="str">
         <v>chromium</v>
       </c>
       <c r="H14" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="15">
@@ -886,13 +886,13 @@
         <v>PASSED</v>
       </c>
       <c r="F15">
-        <v>3.8</v>
+        <v>5.1</v>
       </c>
       <c r="G15" t="str">
         <v>chromium</v>
       </c>
       <c r="H15" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="16">
@@ -912,13 +912,13 @@
         <v>PASSED</v>
       </c>
       <c r="F16">
-        <v>3.5</v>
+        <v>5.3</v>
       </c>
       <c r="G16" t="str">
         <v>chromium</v>
       </c>
       <c r="H16" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="17">
@@ -938,13 +938,13 @@
         <v>PASSED</v>
       </c>
       <c r="F17">
-        <v>4.6</v>
+        <v>6.7</v>
       </c>
       <c r="G17" t="str">
         <v>chromium</v>
       </c>
       <c r="H17" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="18">
@@ -964,13 +964,13 @@
         <v>PASSED</v>
       </c>
       <c r="F18">
-        <v>3.6</v>
+        <v>4.6</v>
       </c>
       <c r="G18" t="str">
         <v>chromium</v>
       </c>
       <c r="H18" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="19">
@@ -990,13 +990,13 @@
         <v>PASSED</v>
       </c>
       <c r="F19">
-        <v>5.9</v>
+        <v>7</v>
       </c>
       <c r="G19" t="str">
         <v>chromium</v>
       </c>
       <c r="H19" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="20">
@@ -1016,13 +1016,13 @@
         <v>PASSED</v>
       </c>
       <c r="F20">
-        <v>4.3</v>
+        <v>4.2</v>
       </c>
       <c r="G20" t="str">
         <v>chromium</v>
       </c>
       <c r="H20" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="21">
@@ -1048,7 +1048,7 @@
         <v>chromium</v>
       </c>
       <c r="H21" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="22">
@@ -1068,13 +1068,13 @@
         <v>PASSED</v>
       </c>
       <c r="F22">
-        <v>4.1</v>
+        <v>4.3</v>
       </c>
       <c r="G22" t="str">
         <v>chromium</v>
       </c>
       <c r="H22" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="23">
@@ -1091,16 +1091,16 @@
         <v>clicking Hired updates status</v>
       </c>
       <c r="E23" t="str">
-        <v>FAILED</v>
+        <v>PASSED</v>
       </c>
       <c r="F23">
-        <v>12.6</v>
+        <v>5.1</v>
       </c>
       <c r="G23" t="str">
         <v>chromium</v>
       </c>
       <c r="H23" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="24">
@@ -1117,16 +1117,16 @@
         <v>clicking Rejected updates status</v>
       </c>
       <c r="E24" t="str">
-        <v>SKIPPED</v>
+        <v>PASSED</v>
       </c>
       <c r="F24">
-        <v>0</v>
+        <v>5.9</v>
       </c>
       <c r="G24" t="str">
         <v>chromium</v>
       </c>
       <c r="H24" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="25">
@@ -1143,16 +1143,16 @@
         <v>status change persists after page refresh</v>
       </c>
       <c r="E25" t="str">
-        <v>SKIPPED</v>
+        <v>PASSED</v>
       </c>
       <c r="F25">
-        <v>0</v>
+        <v>8.3</v>
       </c>
       <c r="G25" t="str">
         <v>chromium</v>
       </c>
       <c r="H25" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="26">
@@ -1172,13 +1172,13 @@
         <v>PASSED</v>
       </c>
       <c r="F26">
-        <v>3.3</v>
+        <v>3.6</v>
       </c>
       <c r="G26" t="str">
         <v>chromium</v>
       </c>
       <c r="H26" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="27">
@@ -1198,13 +1198,13 @@
         <v>PASSED</v>
       </c>
       <c r="F27">
-        <v>3.4</v>
+        <v>3.7</v>
       </c>
       <c r="G27" t="str">
         <v>chromium</v>
       </c>
       <c r="H27" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="28">
@@ -1224,13 +1224,13 @@
         <v>PASSED</v>
       </c>
       <c r="F28">
-        <v>3</v>
+        <v>2.8</v>
       </c>
       <c r="G28" t="str">
         <v>chromium</v>
       </c>
       <c r="H28" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="29">
@@ -1250,13 +1250,13 @@
         <v>PASSED</v>
       </c>
       <c r="F29">
-        <v>3</v>
+        <v>3.1</v>
       </c>
       <c r="G29" t="str">
         <v>chromium</v>
       </c>
       <c r="H29" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="30">
@@ -1276,13 +1276,13 @@
         <v>PASSED</v>
       </c>
       <c r="F30">
-        <v>3.9</v>
+        <v>3.5</v>
       </c>
       <c r="G30" t="str">
         <v>chromium</v>
       </c>
       <c r="H30" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="31">
@@ -1302,13 +1302,13 @@
         <v>PASSED</v>
       </c>
       <c r="F31">
-        <v>2.6</v>
+        <v>4.2</v>
       </c>
       <c r="G31" t="str">
         <v>chromium</v>
       </c>
       <c r="H31" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="32">
@@ -1328,13 +1328,13 @@
         <v>PASSED</v>
       </c>
       <c r="F32">
-        <v>3</v>
+        <v>4.5</v>
       </c>
       <c r="G32" t="str">
         <v>chromium</v>
       </c>
       <c r="H32" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="33">
@@ -1354,13 +1354,13 @@
         <v>PASSED</v>
       </c>
       <c r="F33">
-        <v>1.8</v>
+        <v>4.5</v>
       </c>
       <c r="G33" t="str">
         <v>chromium</v>
       </c>
       <c r="H33" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="34">
@@ -1380,13 +1380,13 @@
         <v>PASSED</v>
       </c>
       <c r="F34">
-        <v>3.1</v>
+        <v>4.3</v>
       </c>
       <c r="G34" t="str">
         <v>chromium</v>
       </c>
       <c r="H34" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="35">
@@ -1406,13 +1406,13 @@
         <v>PASSED</v>
       </c>
       <c r="F35">
-        <v>3.2</v>
+        <v>3.3</v>
       </c>
       <c r="G35" t="str">
         <v>chromium</v>
       </c>
       <c r="H35" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="36">
@@ -1432,13 +1432,13 @@
         <v>PASSED</v>
       </c>
       <c r="F36">
-        <v>3.5</v>
+        <v>3</v>
       </c>
       <c r="G36" t="str">
         <v>chromium</v>
       </c>
       <c r="H36" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="37">
@@ -1458,13 +1458,13 @@
         <v>PASSED</v>
       </c>
       <c r="F37">
-        <v>2.6</v>
+        <v>3.3</v>
       </c>
       <c r="G37" t="str">
         <v>chromium</v>
       </c>
       <c r="H37" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="38">
@@ -1484,13 +1484,13 @@
         <v>PASSED</v>
       </c>
       <c r="F38">
-        <v>1.4</v>
+        <v>1.2</v>
       </c>
       <c r="G38" t="str">
         <v>chromium</v>
       </c>
       <c r="H38" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="39">
@@ -1510,13 +1510,13 @@
         <v>PASSED</v>
       </c>
       <c r="F39">
-        <v>3.3</v>
+        <v>3</v>
       </c>
       <c r="G39" t="str">
         <v>chromium</v>
       </c>
       <c r="H39" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="40">
@@ -1536,13 +1536,13 @@
         <v>PASSED</v>
       </c>
       <c r="F40">
-        <v>1.3</v>
+        <v>1.7</v>
       </c>
       <c r="G40" t="str">
         <v>chromium</v>
       </c>
       <c r="H40" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="41">
@@ -1562,13 +1562,13 @@
         <v>PASSED</v>
       </c>
       <c r="F41">
-        <v>1.7</v>
+        <v>1.9</v>
       </c>
       <c r="G41" t="str">
         <v>chromium</v>
       </c>
       <c r="H41" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="42">
@@ -1588,13 +1588,13 @@
         <v>PASSED</v>
       </c>
       <c r="F42">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
       <c r="G42" t="str">
         <v>chromium</v>
       </c>
       <c r="H42" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="43">
@@ -1614,13 +1614,13 @@
         <v>PASSED</v>
       </c>
       <c r="F43">
-        <v>2.3</v>
+        <v>2.7</v>
       </c>
       <c r="G43" t="str">
         <v>chromium</v>
       </c>
       <c r="H43" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="44">
@@ -1640,13 +1640,13 @@
         <v>PASSED</v>
       </c>
       <c r="F44">
-        <v>3.9</v>
+        <v>3.8</v>
       </c>
       <c r="G44" t="str">
         <v>chromium</v>
       </c>
       <c r="H44" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="45">
@@ -1666,13 +1666,13 @@
         <v>PASSED</v>
       </c>
       <c r="F45">
-        <v>4.2</v>
+        <v>4.7</v>
       </c>
       <c r="G45" t="str">
         <v>chromium</v>
       </c>
       <c r="H45" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="46">
@@ -1692,13 +1692,13 @@
         <v>PASSED</v>
       </c>
       <c r="F46">
-        <v>9.6</v>
+        <v>5.5</v>
       </c>
       <c r="G46" t="str">
         <v>chromium</v>
       </c>
       <c r="H46" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="47">
@@ -1718,13 +1718,13 @@
         <v>PASSED</v>
       </c>
       <c r="F47">
-        <v>4.8</v>
+        <v>1.9</v>
       </c>
       <c r="G47" t="str">
         <v>chromium</v>
       </c>
       <c r="H47" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="48">
@@ -1744,13 +1744,13 @@
         <v>PASSED</v>
       </c>
       <c r="F48">
-        <v>3.5</v>
+        <v>1.6</v>
       </c>
       <c r="G48" t="str">
         <v>chromium</v>
       </c>
       <c r="H48" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="49">
@@ -1770,13 +1770,13 @@
         <v>PASSED</v>
       </c>
       <c r="F49">
-        <v>5.5</v>
+        <v>3.3</v>
       </c>
       <c r="G49" t="str">
         <v>chromium</v>
       </c>
       <c r="H49" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="50">
@@ -1796,13 +1796,13 @@
         <v>PASSED</v>
       </c>
       <c r="F50">
-        <v>6.1</v>
+        <v>4.6</v>
       </c>
       <c r="G50" t="str">
         <v>chromium</v>
       </c>
       <c r="H50" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="51">
@@ -1822,13 +1822,13 @@
         <v>PASSED</v>
       </c>
       <c r="F51">
-        <v>6.5</v>
+        <v>4.7</v>
       </c>
       <c r="G51" t="str">
         <v>chromium</v>
       </c>
       <c r="H51" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="52">
@@ -1848,13 +1848,13 @@
         <v>PASSED</v>
       </c>
       <c r="F52">
-        <v>8.2</v>
+        <v>6.4</v>
       </c>
       <c r="G52" t="str">
         <v>chromium</v>
       </c>
       <c r="H52" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="53">
@@ -1874,13 +1874,13 @@
         <v>PASSED</v>
       </c>
       <c r="F53">
-        <v>6.4</v>
+        <v>5.3</v>
       </c>
       <c r="G53" t="str">
         <v>chromium</v>
       </c>
       <c r="H53" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="54">
@@ -1900,13 +1900,13 @@
         <v>PASSED</v>
       </c>
       <c r="F54">
-        <v>3.6</v>
+        <v>3</v>
       </c>
       <c r="G54" t="str">
         <v>chromium</v>
       </c>
       <c r="H54" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="55">
@@ -1926,13 +1926,13 @@
         <v>PASSED</v>
       </c>
       <c r="F55">
-        <v>2.4</v>
+        <v>1.6</v>
       </c>
       <c r="G55" t="str">
         <v>chromium</v>
       </c>
       <c r="H55" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="56">
@@ -1952,13 +1952,13 @@
         <v>PASSED</v>
       </c>
       <c r="F56">
-        <v>3.3</v>
+        <v>1.8</v>
       </c>
       <c r="G56" t="str">
         <v>chromium</v>
       </c>
       <c r="H56" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="57">
@@ -1978,13 +1978,13 @@
         <v>PASSED</v>
       </c>
       <c r="F57">
-        <v>3.4</v>
+        <v>3.1</v>
       </c>
       <c r="G57" t="str">
         <v>chromium</v>
       </c>
       <c r="H57" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="58">
@@ -2004,13 +2004,13 @@
         <v>PASSED</v>
       </c>
       <c r="F58">
-        <v>3.9</v>
+        <v>3.6</v>
       </c>
       <c r="G58" t="str">
         <v>chromium</v>
       </c>
       <c r="H58" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="59">
@@ -2030,13 +2030,13 @@
         <v>PASSED</v>
       </c>
       <c r="F59">
-        <v>4</v>
+        <v>3.2</v>
       </c>
       <c r="G59" t="str">
         <v>chromium</v>
       </c>
       <c r="H59" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="60">
@@ -2056,13 +2056,13 @@
         <v>PASSED</v>
       </c>
       <c r="F60">
-        <v>3.6</v>
+        <v>2.6</v>
       </c>
       <c r="G60" t="str">
         <v>chromium</v>
       </c>
       <c r="H60" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="61">
@@ -2082,13 +2082,13 @@
         <v>PASSED</v>
       </c>
       <c r="F61">
-        <v>3.6</v>
+        <v>3.1</v>
       </c>
       <c r="G61" t="str">
         <v>chromium</v>
       </c>
       <c r="H61" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="62">
@@ -2108,13 +2108,13 @@
         <v>PASSED</v>
       </c>
       <c r="F62">
-        <v>3.2</v>
+        <v>3</v>
       </c>
       <c r="G62" t="str">
         <v>chromium</v>
       </c>
       <c r="H62" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="63">
@@ -2134,13 +2134,13 @@
         <v>PASSED</v>
       </c>
       <c r="F63">
-        <v>3.6</v>
+        <v>2.6</v>
       </c>
       <c r="G63" t="str">
         <v>chromium</v>
       </c>
       <c r="H63" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="64">
@@ -2160,13 +2160,13 @@
         <v>PASSED</v>
       </c>
       <c r="F64">
-        <v>5.1</v>
+        <v>4.6</v>
       </c>
       <c r="G64" t="str">
         <v>chromium</v>
       </c>
       <c r="H64" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="65">
@@ -2186,13 +2186,13 @@
         <v>PASSED</v>
       </c>
       <c r="F65">
-        <v>2</v>
+        <v>2.3</v>
       </c>
       <c r="G65" t="str">
         <v>chromium</v>
       </c>
       <c r="H65" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="66">
@@ -2212,13 +2212,13 @@
         <v>PASSED</v>
       </c>
       <c r="F66">
-        <v>2</v>
+        <v>3.5</v>
       </c>
       <c r="G66" t="str">
         <v>chromium</v>
       </c>
       <c r="H66" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="67">
@@ -2238,13 +2238,13 @@
         <v>PASSED</v>
       </c>
       <c r="F67">
-        <v>2.2</v>
+        <v>3.7</v>
       </c>
       <c r="G67" t="str">
         <v>chromium</v>
       </c>
       <c r="H67" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="68">
@@ -2264,13 +2264,13 @@
         <v>PASSED</v>
       </c>
       <c r="F68">
-        <v>3.1</v>
+        <v>3.8</v>
       </c>
       <c r="G68" t="str">
         <v>chromium</v>
       </c>
       <c r="H68" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="69">
@@ -2290,13 +2290,13 @@
         <v>PASSED</v>
       </c>
       <c r="F69">
-        <v>4.5</v>
+        <v>7.5</v>
       </c>
       <c r="G69" t="str">
         <v>chromium</v>
       </c>
       <c r="H69" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="70">
@@ -2316,13 +2316,13 @@
         <v>PASSED</v>
       </c>
       <c r="F70">
-        <v>4.3</v>
+        <v>5.5</v>
       </c>
       <c r="G70" t="str">
         <v>chromium</v>
       </c>
       <c r="H70" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="71">
@@ -2342,13 +2342,13 @@
         <v>PASSED</v>
       </c>
       <c r="F71">
-        <v>4.2</v>
+        <v>5.3</v>
       </c>
       <c r="G71" t="str">
         <v>chromium</v>
       </c>
       <c r="H71" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="72">
@@ -2368,13 +2368,13 @@
         <v>PASSED</v>
       </c>
       <c r="F72">
-        <v>4.8</v>
+        <v>6.3</v>
       </c>
       <c r="G72" t="str">
         <v>chromium</v>
       </c>
       <c r="H72" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="73">
@@ -2394,13 +2394,13 @@
         <v>PASSED</v>
       </c>
       <c r="F73">
-        <v>5.5</v>
+        <v>8</v>
       </c>
       <c r="G73" t="str">
         <v>chromium</v>
       </c>
       <c r="H73" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="74">
@@ -2420,13 +2420,13 @@
         <v>PASSED</v>
       </c>
       <c r="F74">
-        <v>4.9</v>
+        <v>5</v>
       </c>
       <c r="G74" t="str">
         <v>chromium</v>
       </c>
       <c r="H74" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="75">
@@ -2446,13 +2446,13 @@
         <v>PASSED</v>
       </c>
       <c r="F75">
-        <v>5.9</v>
+        <v>9.8</v>
       </c>
       <c r="G75" t="str">
         <v>chromium</v>
       </c>
       <c r="H75" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="76">
@@ -2472,13 +2472,13 @@
         <v>PASSED</v>
       </c>
       <c r="F76">
-        <v>4.4</v>
+        <v>5.2</v>
       </c>
       <c r="G76" t="str">
         <v>chromium</v>
       </c>
       <c r="H76" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="77">
@@ -2498,13 +2498,13 @@
         <v>SKIPPED</v>
       </c>
       <c r="F77">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="G77" t="str">
         <v>chromium</v>
       </c>
       <c r="H77" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="78">
@@ -2530,7 +2530,7 @@
         <v>chromium</v>
       </c>
       <c r="H78" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="79">
@@ -2556,7 +2556,7 @@
         <v>chromium</v>
       </c>
       <c r="H79" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="80">
@@ -2576,13 +2576,13 @@
         <v>PASSED</v>
       </c>
       <c r="F80">
-        <v>2.9</v>
+        <v>6.7</v>
       </c>
       <c r="G80" t="str">
         <v>chromium</v>
       </c>
       <c r="H80" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="81">
@@ -2602,13 +2602,13 @@
         <v>PASSED</v>
       </c>
       <c r="F81">
-        <v>3.1</v>
+        <v>4.3</v>
       </c>
       <c r="G81" t="str">
         <v>chromium</v>
       </c>
       <c r="H81" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="82">
@@ -2628,13 +2628,13 @@
         <v>PASSED</v>
       </c>
       <c r="F82">
-        <v>2.8</v>
+        <v>3.7</v>
       </c>
       <c r="G82" t="str">
         <v>chromium</v>
       </c>
       <c r="H82" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="83">
@@ -2654,13 +2654,13 @@
         <v>PASSED</v>
       </c>
       <c r="F83">
-        <v>3</v>
+        <v>3.6</v>
       </c>
       <c r="G83" t="str">
         <v>chromium</v>
       </c>
       <c r="H83" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="84">
@@ -2680,13 +2680,13 @@
         <v>PASSED</v>
       </c>
       <c r="F84">
-        <v>3.4</v>
+        <v>3.5</v>
       </c>
       <c r="G84" t="str">
         <v>chromium</v>
       </c>
       <c r="H84" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="85">
@@ -2706,13 +2706,13 @@
         <v>PASSED</v>
       </c>
       <c r="F85">
-        <v>4.3</v>
+        <v>3.5</v>
       </c>
       <c r="G85" t="str">
         <v>chromium</v>
       </c>
       <c r="H85" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="86">
@@ -2732,13 +2732,13 @@
         <v>PASSED</v>
       </c>
       <c r="F86">
-        <v>3.2</v>
+        <v>3.4</v>
       </c>
       <c r="G86" t="str">
         <v>chromium</v>
       </c>
       <c r="H86" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="87">
@@ -2758,13 +2758,13 @@
         <v>PASSED</v>
       </c>
       <c r="F87">
-        <v>3.2</v>
+        <v>3.7</v>
       </c>
       <c r="G87" t="str">
         <v>chromium</v>
       </c>
       <c r="H87" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="88">
@@ -2784,13 +2784,13 @@
         <v>PASSED</v>
       </c>
       <c r="F88">
-        <v>3.4</v>
+        <v>3.3</v>
       </c>
       <c r="G88" t="str">
         <v>chromium</v>
       </c>
       <c r="H88" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="89">
@@ -2810,13 +2810,13 @@
         <v>PASSED</v>
       </c>
       <c r="F89">
-        <v>4.2</v>
+        <v>5.1</v>
       </c>
       <c r="G89" t="str">
         <v>chromium</v>
       </c>
       <c r="H89" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="90">
@@ -2836,13 +2836,13 @@
         <v>PASSED</v>
       </c>
       <c r="F90">
-        <v>3.6</v>
+        <v>2.6</v>
       </c>
       <c r="G90" t="str">
         <v>chromium</v>
       </c>
       <c r="H90" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="91">
@@ -2862,13 +2862,13 @@
         <v>PASSED</v>
       </c>
       <c r="F91">
-        <v>4.4</v>
+        <v>3.2</v>
       </c>
       <c r="G91" t="str">
         <v>chromium</v>
       </c>
       <c r="H91" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="92">
@@ -2888,13 +2888,13 @@
         <v>PASSED</v>
       </c>
       <c r="F92">
-        <v>6.1</v>
+        <v>4.4</v>
       </c>
       <c r="G92" t="str">
         <v>chromium</v>
       </c>
       <c r="H92" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="93">
@@ -2914,13 +2914,13 @@
         <v>PASSED</v>
       </c>
       <c r="F93">
-        <v>4.5</v>
+        <v>3.7</v>
       </c>
       <c r="G93" t="str">
         <v>chromium</v>
       </c>
       <c r="H93" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="94">
@@ -2940,13 +2940,13 @@
         <v>PASSED</v>
       </c>
       <c r="F94">
-        <v>9</v>
+        <v>8.9</v>
       </c>
       <c r="G94" t="str">
         <v>chromium</v>
       </c>
       <c r="H94" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="95">
@@ -2966,13 +2966,13 @@
         <v>PASSED</v>
       </c>
       <c r="F95">
-        <v>8.5</v>
+        <v>9.3</v>
       </c>
       <c r="G95" t="str">
         <v>chromium</v>
       </c>
       <c r="H95" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="96">
@@ -2992,13 +2992,13 @@
         <v>PASSED</v>
       </c>
       <c r="F96">
-        <v>8.2</v>
+        <v>6.4</v>
       </c>
       <c r="G96" t="str">
         <v>chromium</v>
       </c>
       <c r="H96" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="97">
@@ -3018,13 +3018,13 @@
         <v>PASSED</v>
       </c>
       <c r="F97">
-        <v>2.1</v>
+        <v>1.8</v>
       </c>
       <c r="G97" t="str">
         <v>chromium</v>
       </c>
       <c r="H97" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="98">
@@ -3044,13 +3044,13 @@
         <v>PASSED</v>
       </c>
       <c r="F98">
-        <v>6.6</v>
+        <v>6.8</v>
       </c>
       <c r="G98" t="str">
         <v>chromium</v>
       </c>
       <c r="H98" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="99">
@@ -3070,13 +3070,13 @@
         <v>PASSED</v>
       </c>
       <c r="F99">
-        <v>6.9</v>
+        <v>8.4</v>
       </c>
       <c r="G99" t="str">
         <v>chromium</v>
       </c>
       <c r="H99" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="100">
@@ -3096,13 +3096,13 @@
         <v>PASSED</v>
       </c>
       <c r="F100">
-        <v>6.6</v>
+        <v>8.1</v>
       </c>
       <c r="G100" t="str">
         <v>chromium</v>
       </c>
       <c r="H100" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="101">
@@ -3122,13 +3122,13 @@
         <v>PASSED</v>
       </c>
       <c r="F101">
-        <v>7.2</v>
+        <v>7.9</v>
       </c>
       <c r="G101" t="str">
         <v>chromium</v>
       </c>
       <c r="H101" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="102">
@@ -3148,13 +3148,13 @@
         <v>PASSED</v>
       </c>
       <c r="F102">
-        <v>8.8</v>
+        <v>8.7</v>
       </c>
       <c r="G102" t="str">
         <v>chromium</v>
       </c>
       <c r="H102" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="103">
@@ -3174,13 +3174,13 @@
         <v>PASSED</v>
       </c>
       <c r="F103">
-        <v>10.1</v>
+        <v>7.7</v>
       </c>
       <c r="G103" t="str">
         <v>chromium</v>
       </c>
       <c r="H103" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="104">
@@ -3200,13 +3200,13 @@
         <v>PASSED</v>
       </c>
       <c r="F104">
-        <v>7.8</v>
+        <v>10.2</v>
       </c>
       <c r="G104" t="str">
         <v>chromium</v>
       </c>
       <c r="H104" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="105">
@@ -3226,13 +3226,13 @@
         <v>PASSED</v>
       </c>
       <c r="F105">
-        <v>2.4</v>
+        <v>1.6</v>
       </c>
       <c r="G105" t="str">
         <v>chromium</v>
       </c>
       <c r="H105" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="106">
@@ -3252,13 +3252,13 @@
         <v>PASSED</v>
       </c>
       <c r="F106">
-        <v>8.1</v>
+        <v>8.8</v>
       </c>
       <c r="G106" t="str">
         <v>chromium</v>
       </c>
       <c r="H106" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="107">
@@ -3278,13 +3278,13 @@
         <v>PASSED</v>
       </c>
       <c r="F107">
-        <v>8</v>
+        <v>8.3</v>
       </c>
       <c r="G107" t="str">
         <v>chromium</v>
       </c>
       <c r="H107" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="108">
@@ -3304,13 +3304,13 @@
         <v>PASSED</v>
       </c>
       <c r="F108">
-        <v>1.5</v>
+        <v>1.1</v>
       </c>
       <c r="G108" t="str">
         <v>chromium</v>
       </c>
       <c r="H108" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="109">
@@ -3330,13 +3330,13 @@
         <v>PASSED</v>
       </c>
       <c r="F109">
-        <v>2.5</v>
+        <v>2.3</v>
       </c>
       <c r="G109" t="str">
         <v>chromium</v>
       </c>
       <c r="H109" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="110">
@@ -3356,13 +3356,13 @@
         <v>PASSED</v>
       </c>
       <c r="F110">
-        <v>2.5</v>
+        <v>2.1</v>
       </c>
       <c r="G110" t="str">
         <v>chromium</v>
       </c>
       <c r="H110" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="111">
@@ -3382,13 +3382,13 @@
         <v>PASSED</v>
       </c>
       <c r="F111">
-        <v>2.6</v>
+        <v>2.4</v>
       </c>
       <c r="G111" t="str">
         <v>chromium</v>
       </c>
       <c r="H111" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="112">
@@ -3408,13 +3408,13 @@
         <v>PASSED</v>
       </c>
       <c r="F112">
-        <v>2.6</v>
+        <v>2.8</v>
       </c>
       <c r="G112" t="str">
         <v>chromium</v>
       </c>
       <c r="H112" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="113">
@@ -3434,13 +3434,13 @@
         <v>PASSED</v>
       </c>
       <c r="F113">
-        <v>2.5</v>
+        <v>2.6</v>
       </c>
       <c r="G113" t="str">
         <v>chromium</v>
       </c>
       <c r="H113" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="114">
@@ -3460,13 +3460,13 @@
         <v>PASSED</v>
       </c>
       <c r="F114">
-        <v>2.4</v>
+        <v>3.6</v>
       </c>
       <c r="G114" t="str">
         <v>chromium</v>
       </c>
       <c r="H114" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="115">
@@ -3486,13 +3486,13 @@
         <v>PASSED</v>
       </c>
       <c r="F115">
-        <v>2.7</v>
+        <v>2.3</v>
       </c>
       <c r="G115" t="str">
         <v>chromium</v>
       </c>
       <c r="H115" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="116">
@@ -3512,13 +3512,13 @@
         <v>PASSED</v>
       </c>
       <c r="F116">
-        <v>2.3</v>
+        <v>2.9</v>
       </c>
       <c r="G116" t="str">
         <v>chromium</v>
       </c>
       <c r="H116" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="117">
@@ -3535,16 +3535,16 @@
         <v>applicant count on row matches total count in job detail page</v>
       </c>
       <c r="E117" t="str">
-        <v>FAILED</v>
+        <v>PASSED</v>
       </c>
       <c r="F117">
-        <v>16.2</v>
+        <v>3</v>
       </c>
       <c r="G117" t="str">
         <v>chromium</v>
       </c>
       <c r="H117" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="118">
@@ -3564,13 +3564,13 @@
         <v>PASSED</v>
       </c>
       <c r="F118">
-        <v>2.9</v>
+        <v>3</v>
       </c>
       <c r="G118" t="str">
         <v>chromium</v>
       </c>
       <c r="H118" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="119">
@@ -3590,13 +3590,13 @@
         <v>PASSED</v>
       </c>
       <c r="F119">
-        <v>3.8</v>
+        <v>4</v>
       </c>
       <c r="G119" t="str">
         <v>chromium</v>
       </c>
       <c r="H119" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
     <row r="120">
@@ -3616,13 +3616,13 @@
         <v>PASSED</v>
       </c>
       <c r="F120">
-        <v>3.4</v>
+        <v>5.7</v>
       </c>
       <c r="G120" t="str">
         <v>chromium</v>
       </c>
       <c r="H120" t="str">
-        <v>30/5/2026, 12:02:37 pm</v>
+        <v>1/6/2026, 2:17:07 pm</v>
       </c>
     </row>
   </sheetData>

</xml_diff>